<commit_message>
Sync session16 changes: report keyset comparison, PROD_ITCD filter, output files update
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/upload/S00022_1629_연금저축_미래로기업복지연금보험.xlsx
+++ b/output/upload/S00022_1629_연금저축_미래로기업복지연금보험.xlsx
@@ -1384,7 +1384,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3341,7 +3341,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3929,7 +3929,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -4139,7 +4139,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>162988</t>
+          <t>1629088</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">

</xml_diff>